<commit_message>
Adjust investment cost slightly (+/- 0.5%)
Should prevent different decisions with the same objective function
</commit_message>
<xml_diff>
--- a/data/NREL-118/Power_Storage.xlsx
+++ b/data/NREL-118/Power_Storage.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FelixAuer\Git\LEGO-Pyomo\data\NREL-118\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{015C8960-B869-45D8-A012-A5DD0C8EAB12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18F3BD87-B72E-49EE-975F-F6BBCDEBD55B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-4170" yWindow="-21720" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -502,10 +502,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
+    <numFmt numFmtId="167" formatCode="0.00000"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -519,26 +520,31 @@
       <b/>
       <sz val="11"/>
       <name val="Aptos"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="11"/>
       <name val="Aptos"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Aptos"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="18"/>
       <color rgb="FFFFFFFF"/>
       <name val="Aptos"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Aptos"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="8">
@@ -597,7 +603,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -642,6 +648,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment indent="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1502,7 +1511,7 @@
         <v>1</v>
       </c>
       <c r="R8" s="15">
-        <v>0.1</v>
+        <v>0.10026734851583674</v>
       </c>
       <c r="S8" s="13">
         <v>1</v>
@@ -1511,8 +1520,7 @@
         <v>1</v>
       </c>
       <c r="U8" s="15">
-        <f>2336*1000/100</f>
-        <v>23360</v>
+        <v>23444.980573051093</v>
       </c>
       <c r="V8" s="15">
         <v>0</v>
@@ -1523,8 +1531,8 @@
       <c r="X8" s="16">
         <v>0.96</v>
       </c>
-      <c r="Y8" s="13"/>
-      <c r="Z8" s="13"/>
+      <c r="Y8" s="15"/>
+      <c r="Z8" s="19"/>
       <c r="AA8" s="17"/>
       <c r="AB8" s="17"/>
       <c r="AC8" s="18" t="s">
@@ -1573,7 +1581,7 @@
         <v>1</v>
       </c>
       <c r="R9" s="15">
-        <v>0.1</v>
+        <v>0.10034620903934784</v>
       </c>
       <c r="S9" s="13">
         <v>1</v>
@@ -1582,8 +1590,7 @@
         <v>1</v>
       </c>
       <c r="U9" s="15">
-        <f t="shared" ref="U9:U22" si="0">2336*1000/100</f>
-        <v>23360</v>
+        <v>23353.641585025827</v>
       </c>
       <c r="V9" s="15">
         <v>0</v>
@@ -1594,8 +1601,8 @@
       <c r="X9" s="16">
         <v>0.96</v>
       </c>
-      <c r="Y9" s="13"/>
-      <c r="Z9" s="13"/>
+      <c r="Y9" s="15"/>
+      <c r="Z9" s="19"/>
       <c r="AA9" s="17"/>
       <c r="AB9" s="17"/>
       <c r="AC9" s="18" t="s">
@@ -1644,7 +1651,7 @@
         <v>1</v>
       </c>
       <c r="R10" s="15">
-        <v>0.1</v>
+        <v>0.10016036783568889</v>
       </c>
       <c r="S10" s="13">
         <v>1</v>
@@ -1653,8 +1660,7 @@
         <v>1</v>
       </c>
       <c r="U10" s="15">
-        <f t="shared" si="0"/>
-        <v>23360</v>
+        <v>23326.306738323357</v>
       </c>
       <c r="V10" s="15">
         <v>0</v>
@@ -1665,8 +1671,8 @@
       <c r="X10" s="16">
         <v>0.96</v>
       </c>
-      <c r="Y10" s="13"/>
-      <c r="Z10" s="13"/>
+      <c r="Y10" s="15"/>
+      <c r="Z10" s="19"/>
       <c r="AA10" s="17"/>
       <c r="AB10" s="17"/>
       <c r="AC10" s="18" t="s">
@@ -1715,7 +1721,7 @@
         <v>1</v>
       </c>
       <c r="R11" s="15">
-        <v>0.1</v>
+        <v>0.1000761111765919</v>
       </c>
       <c r="S11" s="13">
         <v>1</v>
@@ -1724,8 +1730,7 @@
         <v>1</v>
       </c>
       <c r="U11" s="15">
-        <f t="shared" si="0"/>
-        <v>23360</v>
+        <v>23389.898989562113</v>
       </c>
       <c r="V11" s="15">
         <v>0</v>
@@ -1736,8 +1741,8 @@
       <c r="X11" s="16">
         <v>0.96</v>
       </c>
-      <c r="Y11" s="13"/>
-      <c r="Z11" s="13"/>
+      <c r="Y11" s="15"/>
+      <c r="Z11" s="19"/>
       <c r="AA11" s="17"/>
       <c r="AB11" s="17"/>
       <c r="AC11" s="18" t="s">
@@ -1786,7 +1791,7 @@
         <v>1</v>
       </c>
       <c r="R12" s="15">
-        <v>0.1</v>
+        <v>0.10034616060067597</v>
       </c>
       <c r="S12" s="13">
         <v>1</v>
@@ -1795,8 +1800,7 @@
         <v>1</v>
       </c>
       <c r="U12" s="15">
-        <f t="shared" si="0"/>
-        <v>23360</v>
+        <v>23297.667140914436</v>
       </c>
       <c r="V12" s="15">
         <v>0</v>
@@ -1807,8 +1811,8 @@
       <c r="X12" s="16">
         <v>0.96</v>
       </c>
-      <c r="Y12" s="13"/>
-      <c r="Z12" s="13"/>
+      <c r="Y12" s="15"/>
+      <c r="Z12" s="19"/>
       <c r="AA12" s="17"/>
       <c r="AB12" s="17"/>
       <c r="AC12" s="18" t="s">
@@ -1857,7 +1861,7 @@
         <v>1</v>
       </c>
       <c r="R13" s="15">
-        <v>0.1</v>
+        <v>9.9925560314092027E-2</v>
       </c>
       <c r="S13" s="13">
         <v>1</v>
@@ -1866,8 +1870,7 @@
         <v>1</v>
       </c>
       <c r="U13" s="15">
-        <f t="shared" si="0"/>
-        <v>23360</v>
+        <v>23360.338127836334</v>
       </c>
       <c r="V13" s="15">
         <v>0</v>
@@ -1878,8 +1881,8 @@
       <c r="X13" s="16">
         <v>0.96</v>
       </c>
-      <c r="Y13" s="13"/>
-      <c r="Z13" s="13"/>
+      <c r="Y13" s="15"/>
+      <c r="Z13" s="19"/>
       <c r="AA13" s="17"/>
       <c r="AB13" s="17"/>
       <c r="AC13" s="18" t="s">
@@ -1928,7 +1931,7 @@
         <v>1</v>
       </c>
       <c r="R14" s="15">
-        <v>0.1</v>
+        <v>0.10008905175849624</v>
       </c>
       <c r="S14" s="13">
         <v>1</v>
@@ -1937,8 +1940,7 @@
         <v>1</v>
       </c>
       <c r="U14" s="15">
-        <f t="shared" si="0"/>
-        <v>23360</v>
+        <v>23473.240277009438</v>
       </c>
       <c r="V14" s="15">
         <v>0</v>
@@ -1949,8 +1951,8 @@
       <c r="X14" s="16">
         <v>0.96</v>
       </c>
-      <c r="Y14" s="13"/>
-      <c r="Z14" s="13"/>
+      <c r="Y14" s="15"/>
+      <c r="Z14" s="19"/>
       <c r="AA14" s="17"/>
       <c r="AB14" s="17"/>
       <c r="AC14" s="18" t="s">
@@ -1999,7 +2001,7 @@
         <v>1</v>
       </c>
       <c r="R15" s="15">
-        <v>0.1</v>
+        <v>0.10048528421709453</v>
       </c>
       <c r="S15" s="13">
         <v>1</v>
@@ -2008,8 +2010,7 @@
         <v>1</v>
       </c>
       <c r="U15" s="15">
-        <f t="shared" si="0"/>
-        <v>23360</v>
+        <v>23379.709150219409</v>
       </c>
       <c r="V15" s="15">
         <v>0</v>
@@ -2020,8 +2021,8 @@
       <c r="X15" s="16">
         <v>0.96</v>
       </c>
-      <c r="Y15" s="13"/>
-      <c r="Z15" s="13"/>
+      <c r="Y15" s="15"/>
+      <c r="Z15" s="19"/>
       <c r="AA15" s="17"/>
       <c r="AB15" s="17"/>
       <c r="AC15" s="18" t="s">
@@ -2070,7 +2071,7 @@
         <v>1</v>
       </c>
       <c r="R16" s="15">
-        <v>0.1</v>
+        <v>9.9778111178256301E-2</v>
       </c>
       <c r="S16" s="13">
         <v>1</v>
@@ -2079,8 +2080,7 @@
         <v>1</v>
       </c>
       <c r="U16" s="15">
-        <f t="shared" si="0"/>
-        <v>23360</v>
+        <v>23462.714021003812</v>
       </c>
       <c r="V16" s="15">
         <v>0</v>
@@ -2091,8 +2091,8 @@
       <c r="X16" s="16">
         <v>0.96</v>
       </c>
-      <c r="Y16" s="13"/>
-      <c r="Z16" s="13"/>
+      <c r="Y16" s="15"/>
+      <c r="Z16" s="19"/>
       <c r="AA16" s="17"/>
       <c r="AB16" s="17"/>
       <c r="AC16" s="18" t="s">
@@ -2141,7 +2141,7 @@
         <v>1</v>
       </c>
       <c r="R17" s="15">
-        <v>0.1</v>
+        <v>9.9582196356760924E-2</v>
       </c>
       <c r="S17" s="13">
         <v>1</v>
@@ -2150,8 +2150,7 @@
         <v>1</v>
       </c>
       <c r="U17" s="15">
-        <f t="shared" si="0"/>
-        <v>23360</v>
+        <v>23437.019117901807</v>
       </c>
       <c r="V17" s="15">
         <v>0</v>
@@ -2162,8 +2161,8 @@
       <c r="X17" s="16">
         <v>0.96</v>
       </c>
-      <c r="Y17" s="13"/>
-      <c r="Z17" s="13"/>
+      <c r="Y17" s="15"/>
+      <c r="Z17" s="19"/>
       <c r="AA17" s="17"/>
       <c r="AB17" s="17"/>
       <c r="AC17" s="18" t="s">
@@ -2212,7 +2211,7 @@
         <v>1</v>
       </c>
       <c r="R18" s="15">
-        <v>0.1</v>
+        <v>9.9766848866623459E-2</v>
       </c>
       <c r="S18" s="13">
         <v>1</v>
@@ -2221,8 +2220,7 @@
         <v>1</v>
       </c>
       <c r="U18" s="15">
-        <f t="shared" si="0"/>
-        <v>23360</v>
+        <v>23338.37077778938</v>
       </c>
       <c r="V18" s="15">
         <v>0</v>
@@ -2233,8 +2231,8 @@
       <c r="X18" s="16">
         <v>0.96</v>
       </c>
-      <c r="Y18" s="13"/>
-      <c r="Z18" s="13"/>
+      <c r="Y18" s="15"/>
+      <c r="Z18" s="19"/>
       <c r="AA18" s="17"/>
       <c r="AB18" s="17"/>
       <c r="AC18" s="18" t="s">
@@ -2283,7 +2281,7 @@
         <v>1</v>
       </c>
       <c r="R19" s="15">
-        <v>0.1</v>
+        <v>9.9830306919604206E-2</v>
       </c>
       <c r="S19" s="13">
         <v>1</v>
@@ -2292,8 +2290,7 @@
         <v>1</v>
       </c>
       <c r="U19" s="15">
-        <f t="shared" si="0"/>
-        <v>23360</v>
+        <v>23282.473552579155</v>
       </c>
       <c r="V19" s="15">
         <v>0</v>
@@ -2304,8 +2301,8 @@
       <c r="X19" s="16">
         <v>0.96</v>
       </c>
-      <c r="Y19" s="13"/>
-      <c r="Z19" s="13"/>
+      <c r="Y19" s="15"/>
+      <c r="Z19" s="19"/>
       <c r="AA19" s="17"/>
       <c r="AB19" s="17"/>
       <c r="AC19" s="18" t="s">
@@ -2354,7 +2351,7 @@
         <v>1</v>
       </c>
       <c r="R20" s="15">
-        <v>0.1</v>
+        <v>0.10029201307129641</v>
       </c>
       <c r="S20" s="13">
         <v>1</v>
@@ -2363,8 +2360,7 @@
         <v>1</v>
       </c>
       <c r="U20" s="15">
-        <f t="shared" si="0"/>
-        <v>23360</v>
+        <v>23462.4378818978</v>
       </c>
       <c r="V20" s="15">
         <v>0</v>
@@ -2375,8 +2371,8 @@
       <c r="X20" s="16">
         <v>0.96</v>
       </c>
-      <c r="Y20" s="13"/>
-      <c r="Z20" s="13"/>
+      <c r="Y20" s="15"/>
+      <c r="Z20" s="19"/>
       <c r="AA20" s="17"/>
       <c r="AB20" s="17"/>
       <c r="AC20" s="18" t="s">
@@ -2425,7 +2421,7 @@
         <v>1</v>
       </c>
       <c r="R21" s="15">
-        <v>0.1</v>
+        <v>0.10002777124959079</v>
       </c>
       <c r="S21" s="13">
         <v>1</v>
@@ -2434,8 +2430,7 @@
         <v>1</v>
       </c>
       <c r="U21" s="15">
-        <f t="shared" si="0"/>
-        <v>23360</v>
+        <v>23325.853660734956</v>
       </c>
       <c r="V21" s="15">
         <v>0</v>
@@ -2446,8 +2441,8 @@
       <c r="X21" s="16">
         <v>0.96</v>
       </c>
-      <c r="Y21" s="13"/>
-      <c r="Z21" s="13"/>
+      <c r="Y21" s="15"/>
+      <c r="Z21" s="19"/>
       <c r="AA21" s="17"/>
       <c r="AB21" s="17"/>
       <c r="AC21" s="18" t="s">
@@ -2496,7 +2491,7 @@
         <v>1</v>
       </c>
       <c r="R22" s="15">
-        <v>0.1</v>
+        <v>9.9890229005466291E-2</v>
       </c>
       <c r="S22" s="13">
         <v>1</v>
@@ -2505,8 +2500,7 @@
         <v>1</v>
       </c>
       <c r="U22" s="15">
-        <f t="shared" si="0"/>
-        <v>23360</v>
+        <v>23389.25735825612</v>
       </c>
       <c r="V22" s="15">
         <v>0</v>
@@ -2517,8 +2511,8 @@
       <c r="X22" s="16">
         <v>0.96</v>
       </c>
-      <c r="Y22" s="13"/>
-      <c r="Z22" s="13"/>
+      <c r="Y22" s="15"/>
+      <c r="Z22" s="19"/>
       <c r="AA22" s="17"/>
       <c r="AB22" s="17"/>
       <c r="AC22" s="18" t="s">

</xml_diff>